<commit_message>
feat: add product, quantity and note fields to invoices
</commit_message>
<xml_diff>
--- a/treasury_master.xlsx
+++ b/treasury_master.xlsx
@@ -52547,7 +52547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52601,6 +52601,21 @@
           <t>created_at</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -52649,6 +52664,11 @@
           <t>2026-04-26</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -52697,6 +52717,11 @@
           <t>2026-04-26</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -52745,6 +52770,11 @@
           <t>2026-04-26</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -52793,6 +52823,11 @@
           <t>2026-04-26</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -52841,6 +52876,11 @@
           <t>2026-04-26</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -52889,6 +52929,11 @@
           <t>2026-04-26</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -52937,6 +52982,11 @@
           <t>2026-04-30</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: fill existing invoices with generic product and quantity data
</commit_message>
<xml_diff>
--- a/treasury_master.xlsx
+++ b/treasury_master.xlsx
@@ -52664,11 +52664,19 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Formation Cloud</t>
+        </is>
+      </c>
       <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Généré automatiquement</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -52717,11 +52725,19 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Licence Logiciel</t>
+        </is>
+      </c>
       <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Généré automatiquement</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -52770,11 +52786,19 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Développement Web</t>
+        </is>
+      </c>
       <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Généré automatiquement</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -52823,11 +52847,19 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Développement Web</t>
+        </is>
+      </c>
       <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Généré automatiquement</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -52876,11 +52908,19 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Abonnement SaaS</t>
+        </is>
+      </c>
       <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Généré automatiquement</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -52929,11 +52969,19 @@
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Hébergement AWS</t>
+        </is>
+      </c>
       <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Généré automatiquement</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -52982,11 +53030,19 @@
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Développement Web</t>
+        </is>
+      </c>
       <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Généré automatiquement</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>